<commit_message>
Add Excel tests for version 1.43 and add missing functionality and tests.
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/test_basketoptions.xlsx
+++ b/tests/workbooktests/workbooks/test_basketoptions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooktests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E357144-259C-4F91-9D20-5623F5B555AB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F70D867B-26B1-4FD6-B2EE-AECAE3F6772C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15105" yWindow="-19605" windowWidth="21915" windowHeight="17220" xr2:uid="{4C44E2F9-E772-4076-A910-7725AADFF688}"/>
+    <workbookView xWindow="-4560" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{4C44E2F9-E772-4076-A910-7725AADFF688}"/>
   </bookViews>
   <sheets>
     <sheet name="Basket option" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,17 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -29,14 +40,14 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
       <extLst>
-        <ext xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray" uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
           <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
         </ext>
       </extLst>
@@ -51,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="52">
   <si>
     <t>Today</t>
   </si>
@@ -201,6 +212,12 @@
   </si>
   <si>
     <t>Himalaya option</t>
+  </si>
+  <si>
+    <t>qlPearsonSpreadEngine</t>
+  </si>
+  <si>
+    <t>qlGaussianCopulaSpreadEngine</t>
   </si>
 </sst>
 </file>
@@ -210,7 +227,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -598,15 +615,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07EF1C03-BB1F-43F7-BF9C-B0202704E6BE}">
-  <dimension ref="A1:F73"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <dimension ref="A1:F77"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="67.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.5703125" customWidth="1"/>
+    <col min="2" max="2" width="67.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -614,7 +631,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -623,7 +640,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -632,7 +649,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R4C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -641,7 +658,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R5C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -650,7 +667,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R6C2BlackVolTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -658,7 +675,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -677,7 +694,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -693,7 +710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -701,7 +718,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -710,7 +727,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R12C2StochasticProcessArray,A</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -719,7 +736,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R15C2PlainVanillaPayoff,A</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -728,7 +745,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R16C2EuropeanExercise,A</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -737,7 +754,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R17C2AmericanExercise,A</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -746,7 +763,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R19C2MinBasketPayoff,A</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -755,7 +772,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R20C2MaxBasketPayoff,A</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -764,7 +781,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R21C2SpreadBasketPayoff,A</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>10</v>
       </c>
@@ -772,12 +789,12 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B24" s="2">
         <v>0.5</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>11</v>
       </c>
@@ -786,12 +803,12 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R25C2AverageBasketPayoff,A</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="15">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -800,7 +817,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R29C2BasketOption,A</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>13</v>
       </c>
@@ -809,7 +826,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R30C2BasketOption,A</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>14</v>
       </c>
@@ -818,7 +835,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R31C2BasketOption,A</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>15</v>
       </c>
@@ -827,12 +844,12 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R32C2BasketOption,A</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="15">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>12</v>
       </c>
@@ -841,7 +858,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R35C2BasketOption,A</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>13</v>
       </c>
@@ -850,7 +867,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R36C2BasketOption,A</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>14</v>
       </c>
@@ -859,7 +876,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R37C2BasketOption,A</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>15</v>
       </c>
@@ -868,12 +885,12 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R38C2BasketOption,A</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>26</v>
       </c>
@@ -881,7 +898,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>28</v>
       </c>
@@ -889,7 +906,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>29</v>
       </c>
@@ -898,7 +915,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="15">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>30</v>
       </c>
@@ -907,7 +924,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R45C2MCLDEuropeanBasketEngine,A</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="15">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>31</v>
       </c>
@@ -916,89 +933,89 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R46C2MCLDAmericanBasketEngine,A</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="15">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>12</v>
       </c>
       <c r="B49" s="6">
         <f t="array" ref="B49">_xll.qlInstrumentNPV(B29,_xll.qlInstrumentSetPricingEngine(B29,$B$45))</f>
-        <v>4.8130399247589892</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2">
+        <v>4.3923285237406091</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>13</v>
       </c>
       <c r="B50" s="6">
         <f t="array" ref="B50">_xll.qlInstrumentNPV(B30,_xll.qlInstrumentSetPricingEngine(B30,$B$45))</f>
-        <v>16.211551395854414</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2">
+        <v>16.6110762398371</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>14</v>
       </c>
       <c r="B51" s="6">
         <f t="array" ref="B51">_xll.qlInstrumentNPV(B31,_xll.qlInstrumentSetPricingEngine(B31,$B$45))</f>
-        <v>9.3903362704326963</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2">
+        <v>9.2694522785816673</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>15</v>
       </c>
       <c r="B52" s="6">
         <f t="array" ref="B52">_xll.qlInstrumentNPV(B32,_xll.qlInstrumentSetPricingEngine(B32,$B$45))</f>
-        <v>9.4099435877230153</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="15">
+        <v>9.3615427541089815</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="55" spans="1:2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>12</v>
       </c>
       <c r="B55" s="6">
         <f t="array" ref="B55">_xll.qlInstrumentNPV(B35,_xll.qlInstrumentSetPricingEngine(B35,$B$46))</f>
-        <v>5.4130659073478027</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2">
+        <v>5.8546994708816609</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>13</v>
       </c>
       <c r="B56" s="6">
         <f t="array" ref="B56">_xll.qlInstrumentNPV(B36,_xll.qlInstrumentSetPricingEngine(B36,$B$46))</f>
-        <v>16.349895189279085</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2">
+        <v>16.302281999965853</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>14</v>
       </c>
       <c r="B57" s="6">
         <f t="array" ref="B57">_xll.qlInstrumentNPV(B37,_xll.qlInstrumentSetPricingEngine(B37,$B$46))</f>
-        <v>8.9475859577728603</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2">
+        <v>9.1238370383810157</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>15</v>
       </c>
       <c r="B58" s="6">
         <f t="array" ref="B58">_xll.qlInstrumentNPV(B38,_xll.qlInstrumentSetPricingEngine(B38,$B$46))</f>
-        <v>9.0959767175743025</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" ht="15">
+        <v>9.3122353469188042</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
         <v>34</v>
       </c>
@@ -1007,7 +1024,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R60C2StulzEngine,A</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="15">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>35</v>
       </c>
@@ -1016,7 +1033,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R61C2BjerksundStenslandSpreadEngine,A</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="15">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
         <v>36</v>
       </c>
@@ -1025,7 +1042,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R62C2OperatorSplittingSpreadEngine,A</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="15">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>37</v>
       </c>
@@ -1034,7 +1051,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R63C2ChoiBasketEngine,A</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="15">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>38</v>
       </c>
@@ -1043,7 +1060,7 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R64C2DengLiZhouBasketEngine,A</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="15">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
         <v>39</v>
       </c>
@@ -1052,63 +1069,99 @@
         <v>欣[test_basketoptions.xlsx]Basket option!R65C2FdndimBlackScholesVanillaEngine,A</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="15">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B66" s="2" t="str" cm="1">
+        <f t="array" ref="B66">_xll.qlPearsonSpreadEngine(B9,B10,B11)</f>
+        <v>欣[test_basketoptions.xlsx]Basket option!R66C2PearsonSpreadEngine,A</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B67" s="2" t="str" cm="1">
+        <f t="array" ref="B67">_xll.qlGaussianCopulaSpreadEngine(B9,B10,B11)</f>
+        <v>欣[test_basketoptions.xlsx]Basket option!R67C2GaussianCopulaSpreadEngine,A</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="68" spans="1:2">
-      <c r="A68" s="7" t="s">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B68" s="6">
-        <f t="array" ref="B68">_xll.qlInstrumentNPV($B$29,_xll.qlInstrumentSetPricingEngine($B$29,B60))</f>
+      <c r="B70" s="6">
+        <f t="array" ref="B70">_xll.qlInstrumentNPV($B$29,_xll.qlInstrumentSetPricingEngine($B$29,B60))</f>
         <v>5.0881276088352108</v>
       </c>
     </row>
-    <row r="69" spans="1:2">
-      <c r="A69" s="7" t="s">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B69" s="6">
-        <f t="array" ref="B69">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B61))</f>
+      <c r="B71" s="6">
+        <f t="array" ref="B71">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B61))</f>
         <v>9.3714474797118879</v>
       </c>
     </row>
-    <row r="70" spans="1:2">
-      <c r="A70" s="7" t="s">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B70" s="6">
-        <f t="array" ref="B70">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B62))</f>
+      <c r="B72" s="6">
+        <f t="array" ref="B72">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B62))</f>
         <v>9.371344349336697</v>
       </c>
     </row>
-    <row r="71" spans="1:2">
-      <c r="A71" s="7" t="s">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B71" s="6">
-        <f t="array" ref="B71">_xll.qlInstrumentNPV($B$32,_xll.qlInstrumentSetPricingEngine($B$32,B63))</f>
+      <c r="B73" s="6">
+        <f t="array" ref="B73">_xll.qlInstrumentNPV($B$32,_xll.qlInstrumentSetPricingEngine($B$32,B63))</f>
         <v>9.4770087612369149</v>
       </c>
     </row>
-    <row r="72" spans="1:2">
-      <c r="A72" s="7" t="s">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B72" s="6">
-        <f t="array" ref="B72">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B64))</f>
+      <c r="B74" s="6">
+        <f t="array" ref="B74">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B64))</f>
         <v>9.3714561400848098</v>
       </c>
     </row>
-    <row r="73" spans="1:2">
-      <c r="A73" s="7" t="s">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B73" s="6">
-        <f t="array" ref="B73">_xll.qlInstrumentNPV($B$30,_xll.qlInstrumentSetPricingEngine($B$30,B65))</f>
+      <c r="B75" s="6">
+        <f t="array" ref="B75">_xll.qlInstrumentNPV($B$30,_xll.qlInstrumentSetPricingEngine($B$30,B65))</f>
         <v>16.43465544034472</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>50</v>
+      </c>
+      <c r="B76" s="6" cm="1">
+        <f t="array" ref="B76">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B66))</f>
+        <v>9.3714564733914134</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>51</v>
+      </c>
+      <c r="B77" s="6" cm="1">
+        <f t="array" ref="B77">_xll.qlInstrumentNPV($B$31,_xll.qlInstrumentSetPricingEngine($B$31,B67))</f>
+        <v>9.3730057504190523</v>
       </c>
     </row>
   </sheetData>
@@ -1120,13 +1173,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58DBCBFC-B212-46DA-8CD3-09A67FA85B1D}">
   <dimension ref="A1:F39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="84.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="84.42578125" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1134,7 +1187,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1143,7 +1196,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1152,7 +1205,7 @@
         <v>欣[test_basketoptions.xlsx]Everest_Himalaya options!R4C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1161,7 +1214,7 @@
         <v>欣[test_basketoptions.xlsx]Everest_Himalaya options!R5C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1170,7 +1223,7 @@
         <v>欣[test_basketoptions.xlsx]Everest_Himalaya options!R6C2BlackVolTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1178,7 +1231,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1197,7 +1250,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1213,7 +1266,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -1221,7 +1274,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -1230,7 +1283,7 @@
         <v>欣[test_basketoptions.xlsx]Everest_Himalaya options!R12C2StochasticProcessArray,A</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1239,7 +1292,7 @@
         <v>欣[test_basketoptions.xlsx]Everest_Himalaya options!R14C2EuropeanExercise,A</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -1247,7 +1300,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>41</v>
       </c>
@@ -1255,7 +1308,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>42</v>
       </c>
@@ -1264,7 +1317,7 @@
         <v>欣[test_basketoptions.xlsx]Everest_Himalaya options!R19C2EverestOption,A</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -1273,33 +1326,33 @@
         <v>欣[test_basketoptions.xlsx]Everest_Himalaya options!R21C2Schedule,A</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B22" s="1" cm="1">
         <f t="array" ref="B22:B26">_xll.qlScheduleDates(B21)</f>
         <v>46174</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B23" s="1">
         <v>46266</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B24" s="1">
         <v>46357</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B25" s="1">
         <v>46447</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B26" s="1">
         <v>46539</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>44</v>
       </c>
@@ -1307,7 +1360,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="15">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>45</v>
       </c>
@@ -1316,12 +1369,12 @@
         <v>欣[test_basketoptions.xlsx]Everest_Himalaya options!R28C2HimalayaOption,A</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="15">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>26</v>
       </c>
@@ -1329,7 +1382,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>28</v>
       </c>
@@ -1337,7 +1390,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>29</v>
       </c>
@@ -1346,7 +1399,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="15">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>46</v>
       </c>
@@ -1355,7 +1408,7 @@
         <v>欣[test_basketoptions.xlsx]Everest_Himalaya options!R34C2MCLDEverestEngine,A</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="15">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>47</v>
       </c>
@@ -1364,21 +1417,21 @@
         <v>欣[test_basketoptions.xlsx]Everest_Himalaya options!R35C2MCLDHimalayaEngine,A</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="15">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>48</v>
       </c>
       <c r="B38" s="4" cm="1">
         <f t="array" ref="B38">_xll.qlInstrumentNPV(B19,_xll.qlInstrumentSetPricingEngine(B19,B34))</f>
-        <v>574.2923657082772</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2">
+        <v>574.52201425851081</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>49</v>
       </c>

</xml_diff>